<commit_message>
+ added publication for cdlFN26
</commit_message>
<xml_diff>
--- a/List of Kinetic Models.xlsx
+++ b/List of Kinetic Models.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dropbox\MyProjects\kinmodre\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{983BD7FF-7989-4A58-90E3-C6FFDF1D3E11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FCD4FA1D-E1F6-40C9-B2CA-173A1EAC784A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{A48245FD-6B6A-497E-8B16-C1CADEA3146F}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="129">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="130">
   <si>
     <t>Model Name</t>
   </si>
@@ -595,6 +595,9 @@
   </si>
   <si>
     <t>Modankap et al. (2026) Ab Initio Whole Cell Kinetic Model of Bifidobacterium longum subsp. longum JCM1217 (blmSHM26). American Journal of Pathology &amp; Research 5(8): 1-5.</t>
+  </si>
+  <si>
+    <t>Ng et al. 2026. Ab Initio Whole Cell Kinetic Model of Clostridioides difficile R20291 (cdlFN26). International Journal of Translational Science &amp; Reseearch 2(3): 1-4.</t>
   </si>
 </sst>
 </file>
@@ -1356,7 +1359,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:8" ht="31" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
         <v>118</v>
       </c>
@@ -1377,6 +1380,9 @@
       </c>
       <c r="G10" s="2">
         <v>880</v>
+      </c>
+      <c r="H10" s="4" t="s">
+        <v>129</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="31" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
+ added publication for cglTY26
</commit_message>
<xml_diff>
--- a/List of Kinetic Models.xlsx
+++ b/List of Kinetic Models.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dropbox\MyProjects\kinmodre\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FCD4FA1D-E1F6-40C9-B2CA-173A1EAC784A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92AB79EC-4666-416C-A5C4-AE0DF7569402}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{A48245FD-6B6A-497E-8B16-C1CADEA3146F}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="130">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="149" uniqueCount="131">
   <si>
     <t>Model Name</t>
   </si>
@@ -598,6 +598,9 @@
   </si>
   <si>
     <t>Ng et al. 2026. Ab Initio Whole Cell Kinetic Model of Clostridioides difficile R20291 (cdlFN26). International Journal of Translational Science &amp; Reseearch 2(3): 1-4.</t>
+  </si>
+  <si>
+    <t>Lim et al. 2026. Ab Initio Whole Cell Kinetic Model of Multi-strain Corynebacterium glutamicum (cglTY26). American Journal of Medical and Clinical Research &amp; Reviews 5(9): 1-8.</t>
   </si>
 </sst>
 </file>
@@ -2006,7 +2009,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:8" ht="31" x14ac:dyDescent="0.35">
       <c r="A35" s="2" t="s">
         <v>122</v>
       </c>
@@ -2027,6 +2030,9 @@
       </c>
       <c r="G35" s="2">
         <v>1109</v>
+      </c>
+      <c r="H35" s="4" t="s">
+        <v>130</v>
       </c>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
+ added publication for bbrdPS26
</commit_message>
<xml_diff>
--- a/List of Kinetic Models.xlsx
+++ b/List of Kinetic Models.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dropbox\MyProjects\kinmodre\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92AB79EC-4666-416C-A5C4-AE0DF7569402}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9FA65F4A-916A-4A94-A083-4727EB72FEEB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{A48245FD-6B6A-497E-8B16-C1CADEA3146F}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="149" uniqueCount="131">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="132">
   <si>
     <t>Model Name</t>
   </si>
@@ -601,6 +601,9 @@
   </si>
   <si>
     <t>Lim et al. 2026. Ab Initio Whole Cell Kinetic Model of Multi-strain Corynebacterium glutamicum (cglTY26). American Journal of Medical and Clinical Research &amp; Reviews 5(9): 1-8.</t>
+  </si>
+  <si>
+    <t>Subramanian et al. (2026) Ab Initio Whole Cell Kinetic Model of Bifidobacterium breve DSM 20213 (bbrdPS26). Journal of Clinical Immunology &amp; Microbiology 7(3):1-6.</t>
   </si>
 </sst>
 </file>
@@ -1960,7 +1963,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:8" ht="31" x14ac:dyDescent="0.35">
       <c r="A33" s="2" t="s">
         <v>126</v>
       </c>
@@ -1981,6 +1984,9 @@
       </c>
       <c r="G33" s="2">
         <v>453</v>
+      </c>
+      <c r="H33" s="4" t="s">
+        <v>131</v>
       </c>
     </row>
     <row r="34" spans="1:8" ht="31" x14ac:dyDescent="0.35">

</xml_diff>